<commit_message>
Fixed identity schema json
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/identity_schema.xlsx
+++ b/mosip_master/xlsx/identity_schema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\eclipse-workspace\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3F5598-810E-4413-B385-5A3125208622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7C1BCB-805B-4E3F-87C6-5A2E980F3BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -154,6 +154,8 @@
 				"surname",
 				"dateOfBirth",
 				"gender",
+				"countryOfCitizenship",
+				"maritalStatus",
 				"addressLine1",
 				"addressLine2",
 				"island",
@@ -295,7 +297,8 @@
 					"fieldCategory": "pvt",
 					"format": "none",
 					"type": "string",
-					"fieldType": "default"
+					"fieldType": "default",
+					"$ref": "#\/definitions\/simpleType"
 				},
 				"maritalStatus": {
 					"bioAttributes": [
@@ -489,7 +492,8 @@
 					"fieldCategory": "kyc",
 					"format": "none",
 					"type": "string",
-					"fieldType": "default"
+					"fieldType": "default",
+					"$ref": "#/definitions/simpleType"
 				},
 				"passportDateOfIssue": {
 					"bioAttributes": [

</xml_diff>